<commit_message>
Add SOH report triggered by container bill webhook
</commit_message>
<xml_diff>
--- a/reports/SOH_17_09_2026.xlsx
+++ b/reports/SOH_17_09_2026.xlsx
@@ -909,7 +909,7 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>-69</v>
+        <v>-81</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>8000</v>
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>21000</v>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>0</v>
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>423</v>
+        <v>438</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>21000</v>
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>-48</v>
+        <v>-75</v>
       </c>
       <c r="E22" s="3" t="n">
         <v>8000</v>
@@ -1133,7 +1133,7 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E25" s="3" t="n">
         <v>40000</v>
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>983</v>
+        <v>953</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>40000</v>
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>1467</v>
+        <v>1446</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>17000</v>
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>804</v>
+        <v>798</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>10500</v>
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>224</v>
+        <v>206</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>40000</v>
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>535</v>
+        <v>523</v>
       </c>
       <c r="E35" s="3" t="n">
         <v>10500</v>
@@ -1441,7 +1441,7 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="E36" s="3" t="n">
         <v>10500</v>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>48000</v>
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="E38" s="3" t="n">
         <v>24000</v>
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>10500</v>
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>1104</v>
+        <v>1102</v>
       </c>
       <c r="E44" s="3" t="n">
         <v>4500</v>
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>1178</v>
+        <v>1172</v>
       </c>
       <c r="E45" s="3" t="n">
         <v>12500</v>
@@ -1805,7 +1805,7 @@
         </is>
       </c>
       <c r="D49" s="2" t="n">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E49" s="3" t="n">
         <v>81000</v>
@@ -1833,7 +1833,7 @@
         </is>
       </c>
       <c r="D50" s="2" t="n">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="E50" s="3" t="n">
         <v>81000</v>
@@ -1861,7 +1861,7 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="E51" s="3" t="n">
         <v>81000</v>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>814</v>
+        <v>795</v>
       </c>
       <c r="E57" s="3" t="n">
         <v>51000</v>
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>1671</v>
+        <v>1655</v>
       </c>
       <c r="E59" s="3" t="n">
         <v>51000</v>
@@ -2113,7 +2113,7 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>384</v>
+        <v>370</v>
       </c>
       <c r="E60" s="3" t="n">
         <v>26500</v>
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>1251</v>
+        <v>1222</v>
       </c>
       <c r="E62" s="3" t="n">
         <v>51000</v>
@@ -2197,7 +2197,7 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="E63" s="3" t="n">
         <v>26500</v>
@@ -2225,7 +2225,7 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>222</v>
+        <v>200</v>
       </c>
       <c r="E64" s="3" t="n">
         <v>26500</v>
@@ -2337,7 +2337,7 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="E68" s="3" t="n">
         <v>26500</v>
@@ -2505,7 +2505,7 @@
         </is>
       </c>
       <c r="D74" s="2" t="n">
-        <v>1479</v>
+        <v>1476</v>
       </c>
       <c r="E74" s="3" t="n">
         <v>3000</v>
@@ -2533,7 +2533,7 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>804</v>
+        <v>777</v>
       </c>
       <c r="E75" s="3" t="n">
         <v>4000</v>
@@ -2561,7 +2561,7 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E76" s="3" t="n">
         <v>4000</v>
@@ -2589,7 +2589,7 @@
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>1266</v>
+        <v>1264</v>
       </c>
       <c r="E77" s="3" t="n">
         <v>3000</v>
@@ -2813,7 +2813,7 @@
         </is>
       </c>
       <c r="D85" s="2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E85" s="3" t="n">
         <v>20000</v>
@@ -2925,7 +2925,7 @@
         </is>
       </c>
       <c r="D89" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E89" s="3" t="n">
         <v>31000</v>
@@ -3009,7 +3009,7 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>1673</v>
+        <v>1667</v>
       </c>
       <c r="E92" s="3" t="n">
         <v>8000</v>
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>252</v>
+        <v>228</v>
       </c>
       <c r="E93" s="3" t="n">
         <v>8000</v>
@@ -3121,7 +3121,7 @@
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E96" s="3" t="n">
         <v>8000</v>
@@ -3177,7 +3177,7 @@
         </is>
       </c>
       <c r="D98" s="2" t="n">
-        <v>518</v>
+        <v>512</v>
       </c>
       <c r="E98" s="3" t="n">
         <v>8597</v>
@@ -3373,7 +3373,7 @@
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="E105" s="3" t="n">
         <v>4708</v>
@@ -3429,7 +3429,7 @@
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E107" s="3" t="n">
         <v>1</v>
@@ -3485,7 +3485,7 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>3068</v>
+        <v>3055</v>
       </c>
       <c r="E109" s="3" t="n">
         <v>3876</v>
@@ -3513,7 +3513,7 @@
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>3073</v>
+        <v>3048</v>
       </c>
       <c r="E110" s="3" t="n">
         <v>3500</v>
@@ -3541,7 +3541,7 @@
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="E111" s="3" t="n">
         <v>25000</v>
@@ -3569,7 +3569,7 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="E112" s="3" t="n">
         <v>25000</v>
@@ -3625,7 +3625,7 @@
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="E114" s="3" t="n">
         <v>36000</v>
@@ -3681,7 +3681,7 @@
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>487</v>
+        <v>481</v>
       </c>
       <c r="E116" s="3" t="n">
         <v>36000</v>
@@ -3765,7 +3765,7 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>151</v>
+        <v>115</v>
       </c>
       <c r="E119" s="3" t="n">
         <v>5000</v>
@@ -3901,7 +3901,7 @@
         </is>
       </c>
       <c r="D124" s="2" t="n">
-        <v>-28</v>
+        <v>-36</v>
       </c>
       <c r="E124" s="3" t="n">
         <v>7000</v>
@@ -3957,7 +3957,7 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>5904</v>
+        <v>5688</v>
       </c>
       <c r="E126" s="3" t="n">
         <v>2500</v>
@@ -4013,7 +4013,7 @@
         </is>
       </c>
       <c r="D128" s="2" t="n">
-        <v>1557</v>
+        <v>1341</v>
       </c>
       <c r="E128" s="3" t="n">
         <v>3500</v>
@@ -4041,7 +4041,7 @@
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="E129" s="3" t="n">
         <v>2500</v>
@@ -4125,7 +4125,7 @@
         </is>
       </c>
       <c r="D132" s="2" t="n">
-        <v>-28</v>
+        <v>-34</v>
       </c>
       <c r="E132" s="3" t="n">
         <v>8000</v>
@@ -4153,7 +4153,7 @@
         </is>
       </c>
       <c r="D133" s="2" t="n">
-        <v>-28</v>
+        <v>-40</v>
       </c>
       <c r="E133" s="3" t="n">
         <v>5000</v>
@@ -4209,7 +4209,7 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>1377</v>
+        <v>1161</v>
       </c>
       <c r="E135" s="3" t="n">
         <v>2500</v>
@@ -4265,7 +4265,7 @@
         </is>
       </c>
       <c r="D137" s="2" t="n">
-        <v>1153</v>
+        <v>937</v>
       </c>
       <c r="E137" s="3" t="n">
         <v>3500</v>
@@ -4713,7 +4713,7 @@
         </is>
       </c>
       <c r="D153" s="2" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E153" s="3" t="n">
         <v>1</v>
@@ -4769,7 +4769,7 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E155" s="3" t="n">
         <v>1</v>
@@ -4797,7 +4797,7 @@
         </is>
       </c>
       <c r="D156" s="2" t="n">
-        <v>1082</v>
+        <v>1070</v>
       </c>
       <c r="E156" s="3" t="n">
         <v>26000</v>
@@ -4881,7 +4881,7 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>545</v>
+        <v>541</v>
       </c>
       <c r="E159" s="3" t="n">
         <v>1</v>
@@ -5285,7 +5285,7 @@
         </is>
       </c>
       <c r="D174" s="2" t="n">
-        <v>1107</v>
+        <v>1104</v>
       </c>
       <c r="E174" s="3" t="n">
         <v>13500</v>
@@ -5365,7 +5365,7 @@
         </is>
       </c>
       <c r="D177" s="2" t="n">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="E177" s="3" t="n">
         <v>1</v>
@@ -6177,7 +6177,7 @@
         </is>
       </c>
       <c r="D207" s="2" t="n">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E207" s="3" t="n">
         <v>1</v>
@@ -6685,7 +6685,7 @@
         </is>
       </c>
       <c r="D226" s="2" t="n">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="E226" s="3" t="n">
         <v>1</v>
@@ -8393,7 +8393,7 @@
         </is>
       </c>
       <c r="D288" s="2" t="n">
-        <v>1650</v>
+        <v>1626</v>
       </c>
       <c r="E288" s="3" t="n">
         <v>7347</v>
@@ -9485,7 +9485,7 @@
         </is>
       </c>
       <c r="D327" s="2" t="n">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="E327" s="3" t="n">
         <v>23219</v>
@@ -9766,7 +9766,7 @@
         </is>
       </c>
       <c r="D337" s="2" t="n">
-        <v>1245</v>
+        <v>1209</v>
       </c>
       <c r="E337" s="3" t="n">
         <v>9872</v>
@@ -9794,7 +9794,7 @@
         </is>
       </c>
       <c r="D338" s="2" t="n">
-        <v>1829</v>
+        <v>1813</v>
       </c>
       <c r="E338" s="3" t="n">
         <v>10170</v>
@@ -11502,7 +11502,7 @@
         </is>
       </c>
       <c r="D399" s="2" t="n">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="E399" s="3" t="n">
         <v>5980</v>
@@ -12454,7 +12454,7 @@
         </is>
       </c>
       <c r="D433" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E433" s="3" t="n">
         <v>5998</v>
@@ -12622,7 +12622,7 @@
         </is>
       </c>
       <c r="D439" s="2" t="n">
-        <v>161</v>
+        <v>137</v>
       </c>
       <c r="E439" s="3" t="n">
         <v>8552</v>
@@ -12818,7 +12818,7 @@
         </is>
       </c>
       <c r="D446" s="2" t="n">
-        <v>163</v>
+        <v>139</v>
       </c>
       <c r="E446" s="3" t="n">
         <v>8734</v>
@@ -13182,7 +13182,7 @@
         </is>
       </c>
       <c r="D459" s="2" t="n">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E459" s="3" t="n">
         <v>9544</v>
@@ -13994,7 +13994,7 @@
         </is>
       </c>
       <c r="D488" s="2" t="n">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="E488" s="3" t="n">
         <v>41871</v>
@@ -14974,7 +14974,7 @@
         </is>
       </c>
       <c r="D523" s="2" t="n">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="E523" s="3" t="n">
         <v>6593</v>
@@ -17523,7 +17523,7 @@
         </is>
       </c>
       <c r="D614" s="2" t="n">
-        <v>2866</v>
+        <v>2626</v>
       </c>
       <c r="E614" s="3" t="n">
         <v>10251</v>
@@ -17551,7 +17551,7 @@
         </is>
       </c>
       <c r="D615" s="2" t="n">
-        <v>1320</v>
+        <v>1224</v>
       </c>
       <c r="E615" s="3" t="n">
         <v>12094</v>
@@ -17719,7 +17719,7 @@
         </is>
       </c>
       <c r="D621" s="2" t="n">
-        <v>103</v>
+        <v>79</v>
       </c>
       <c r="E621" s="3" t="n">
         <v>30087</v>
@@ -18251,7 +18251,7 @@
         </is>
       </c>
       <c r="D640" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E640" s="3" t="n">
         <v>8552</v>
@@ -19147,7 +19147,7 @@
         </is>
       </c>
       <c r="D672" s="2" t="n">
-        <v>1439</v>
+        <v>1391</v>
       </c>
       <c r="E672" s="3" t="n">
         <v>5110</v>
@@ -21723,7 +21723,7 @@
         </is>
       </c>
       <c r="D764" s="2" t="n">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E764" s="3" t="n">
         <v>6934</v>
@@ -21751,7 +21751,7 @@
         </is>
       </c>
       <c r="D765" s="2" t="n">
-        <v>802</v>
+        <v>794</v>
       </c>
       <c r="E765" s="3" t="n">
         <v>7465</v>
@@ -23600,7 +23600,7 @@
         </is>
       </c>
       <c r="D831" s="2" t="n">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="E831" s="3" t="n">
         <v>6718</v>
@@ -23628,7 +23628,7 @@
         </is>
       </c>
       <c r="D832" s="2" t="n">
-        <v>1525</v>
+        <v>1501</v>
       </c>
       <c r="E832" s="3" t="n">
         <v>14096</v>
@@ -24469,7 +24469,7 @@
         </is>
       </c>
       <c r="D862" s="2" t="n">
-        <v>759</v>
+        <v>687</v>
       </c>
       <c r="E862" s="3" t="n">
         <v>8181</v>
@@ -28308,7 +28308,7 @@
         </is>
       </c>
       <c r="D999" s="2" t="n">
-        <v>296</v>
+        <v>284</v>
       </c>
       <c r="E999" s="3" t="n">
         <v>14215</v>
@@ -28392,7 +28392,7 @@
         </is>
       </c>
       <c r="D1002" s="2" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="E1002" s="3" t="n">
         <v>11261</v>
@@ -28840,7 +28840,7 @@
         </is>
       </c>
       <c r="D1018" s="2" t="n">
-        <v>786</v>
+        <v>714</v>
       </c>
       <c r="E1018" s="3" t="n">
         <v>8060</v>
@@ -29513,7 +29513,7 @@
         </is>
       </c>
       <c r="D1042" s="2" t="n">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="E1042" s="3" t="n">
         <v>8402</v>
@@ -29821,7 +29821,7 @@
         </is>
       </c>
       <c r="D1053" s="2" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E1053" s="3" t="n">
         <v>32068</v>
@@ -30045,7 +30045,7 @@
         </is>
       </c>
       <c r="D1061" s="2" t="n">
-        <v>121</v>
+        <v>97</v>
       </c>
       <c r="E1061" s="3" t="n">
         <v>10691</v>
@@ -30269,7 +30269,7 @@
         </is>
       </c>
       <c r="D1069" s="2" t="n">
-        <v>91</v>
+        <v>61</v>
       </c>
       <c r="E1069" s="3" t="n">
         <v>18503</v>
@@ -30745,7 +30745,7 @@
         </is>
       </c>
       <c r="D1086" s="2" t="n">
-        <v>1257</v>
+        <v>1233</v>
       </c>
       <c r="E1086" s="3" t="n">
         <v>5086</v>
@@ -31277,7 +31277,7 @@
         </is>
       </c>
       <c r="D1105" s="2" t="n">
-        <v>624</v>
+        <v>600</v>
       </c>
       <c r="E1105" s="3" t="n">
         <v>11372</v>
@@ -32649,7 +32649,7 @@
         </is>
       </c>
       <c r="D1154" s="2" t="n">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="E1154" s="3" t="n">
         <v>6249</v>
@@ -32705,7 +32705,7 @@
         </is>
       </c>
       <c r="D1156" s="2" t="n">
-        <v>103</v>
+        <v>55</v>
       </c>
       <c r="E1156" s="3" t="n">
         <v>24480</v>
@@ -32789,7 +32789,7 @@
         </is>
       </c>
       <c r="D1159" s="2" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E1159" s="3" t="n">
         <v>4831</v>
@@ -33293,7 +33293,7 @@
         </is>
       </c>
       <c r="D1177" s="2" t="n">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="E1177" s="3" t="n">
         <v>14554</v>
@@ -33937,7 +33937,7 @@
         </is>
       </c>
       <c r="D1200" s="2" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E1200" s="3" t="n">
         <v>5601</v>
@@ -34917,7 +34917,7 @@
         </is>
       </c>
       <c r="D1235" s="2" t="n">
-        <v>184</v>
+        <v>160</v>
       </c>
       <c r="E1235" s="3" t="n">
         <v>5671</v>
@@ -36569,7 +36569,7 @@
         </is>
       </c>
       <c r="D1294" s="2" t="n">
-        <v>268</v>
+        <v>244</v>
       </c>
       <c r="E1294" s="3" t="n">
         <v>12722</v>
@@ -37325,7 +37325,7 @@
         </is>
       </c>
       <c r="D1321" s="2" t="n">
-        <v>330</v>
+        <v>300</v>
       </c>
       <c r="E1321" s="3" t="n">
         <v>7139</v>
@@ -37521,7 +37521,7 @@
         </is>
       </c>
       <c r="D1328" s="2" t="n">
-        <v>1181</v>
+        <v>1145</v>
       </c>
       <c r="E1328" s="3" t="n">
         <v>7174</v>
@@ -38109,7 +38109,7 @@
         </is>
       </c>
       <c r="D1349" s="2" t="n">
-        <v>461</v>
+        <v>431</v>
       </c>
       <c r="E1349" s="3" t="n">
         <v>14093</v>
@@ -38277,7 +38277,7 @@
         </is>
       </c>
       <c r="D1355" s="2" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="E1355" s="3" t="n">
         <v>10487</v>
@@ -38473,7 +38473,7 @@
         </is>
       </c>
       <c r="D1362" s="2" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E1362" s="3" t="n">
         <v>18059</v>
@@ -38501,7 +38501,7 @@
         </is>
       </c>
       <c r="D1363" s="2" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="E1363" s="3" t="n">
         <v>7068</v>
@@ -39621,7 +39621,7 @@
         </is>
       </c>
       <c r="D1403" s="2" t="n">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="E1403" s="3" t="n">
         <v>9007</v>
@@ -39649,7 +39649,7 @@
         </is>
       </c>
       <c r="D1404" s="2" t="n">
-        <v>2537</v>
+        <v>2513</v>
       </c>
       <c r="E1404" s="3" t="n">
         <v>11094</v>
@@ -39677,7 +39677,7 @@
         </is>
       </c>
       <c r="D1405" s="2" t="n">
-        <v>1068</v>
+        <v>1056</v>
       </c>
       <c r="E1405" s="3" t="n">
         <v>10548</v>
@@ -39705,7 +39705,7 @@
         </is>
       </c>
       <c r="D1406" s="2" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="E1406" s="3" t="n">
         <v>15697</v>
@@ -39845,7 +39845,7 @@
         </is>
       </c>
       <c r="D1411" s="2" t="n">
-        <v>441</v>
+        <v>435</v>
       </c>
       <c r="E1411" s="3" t="n">
         <v>8626</v>
@@ -41133,7 +41133,7 @@
         </is>
       </c>
       <c r="D1457" s="2" t="n">
-        <v>485</v>
+        <v>479</v>
       </c>
       <c r="E1457" s="3" t="n">
         <v>15250</v>
@@ -41161,7 +41161,7 @@
         </is>
       </c>
       <c r="D1458" s="2" t="n">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="E1458" s="3" t="n">
         <v>9428</v>
@@ -41189,7 +41189,7 @@
         </is>
       </c>
       <c r="D1459" s="2" t="n">
-        <v>459</v>
+        <v>453</v>
       </c>
       <c r="E1459" s="3" t="n">
         <v>11283</v>
@@ -41497,7 +41497,7 @@
         </is>
       </c>
       <c r="D1470" s="2" t="n">
-        <v>464</v>
+        <v>286</v>
       </c>
       <c r="E1470" s="3" t="n">
         <v>4836</v>
@@ -41525,7 +41525,7 @@
         </is>
       </c>
       <c r="D1471" s="2" t="n">
-        <v>2486</v>
+        <v>2462</v>
       </c>
       <c r="E1471" s="3" t="n">
         <v>7312</v>
@@ -42365,7 +42365,7 @@
         </is>
       </c>
       <c r="D1501" s="2" t="n">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="E1501" s="3" t="n">
         <v>12491</v>
@@ -44047,7 +44047,7 @@
         </is>
       </c>
       <c r="D1561" s="2" t="n">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="E1561" s="3" t="n">
         <v>11606</v>
@@ -44243,7 +44243,7 @@
         </is>
       </c>
       <c r="D1568" s="2" t="n">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E1568" s="3" t="n">
         <v>20776</v>

</xml_diff>